<commit_message>
Events: correct UTC-shifted export dates from local xlsx; fix two roster dates
</commit_message>
<xml_diff>
--- a/Cerebral/config/audience_event_mapping.xlsx
+++ b/Cerebral/config/audience_event_mapping.xlsx
@@ -116,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -150,6 +150,9 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -754,19 +757,17 @@
       <c r="F5" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>2025-08-24</t>
-        </is>
+      <c r="G5" s="15" t="n">
+        <v>45892</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Planet Brooklyn 2-day Music Festival (day 2)</t>
+          <t>Planet Brooklyn 2-day Music Festival</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>DTBK</t>
+          <t>Not In Store</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -2039,14 +2040,12 @@
       <c r="F26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
+      <c r="G26" s="14" t="n">
+        <v>46181</v>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>Tray Tables Up June (calendar shows 06-08)</t>
+          <t>TRAY TABLES UP w. Litclub Founder, Kelly</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">

</xml_diff>